<commit_message>
Fix IPO market cap
</commit_message>
<xml_diff>
--- a/ipo_watch_results.xlsx
+++ b/ipo_watch_results.xlsx
@@ -671,7 +671,7 @@
       <c r="L3" t="inlineStr"/>
       <c r="M3" t="inlineStr">
         <is>
-          <t>460억</t>
+          <t>1222억</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>1874억</t>
+          <t>1876억</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">

</xml_diff>